<commit_message>
@ Add dynamic Excel import to setup
- Add tab UI for switching between Setup Default and Import Excel
- Add drag & drop file upload for .xlsx and .csv files
- Auto-detect column types (INTEGER, DOUBLE, BOOLEAN, TIMESTAMP, TEXT)
- Generate CREATE TABLE SQL based on Excel headers
- Batch insert data (100 rows per batch)
- DROP existing table before creating new one

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
@
</commit_message>
<xml_diff>
--- a/Alokasi_Petugas.xlsx
+++ b/Alokasi_Petugas.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rifah\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rifah\Downloads\SE2026-Tempuran-master\SE2026-Tempuran-master\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D30F2CA-53DF-4F2F-ACF3-BF774AFAF0FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36A9BDB0-835A-4C67-A719-91FF66AE0E28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DE4ED9FF-8DCB-49D4-9C3D-FE28C890E50C}"/>
   </bookViews>

</xml_diff>